<commit_message>
update new version + add sound
</commit_message>
<xml_diff>
--- a/questions.xlsx
+++ b/questions.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000"/>
+    <workbookView windowWidth="11520" windowHeight="8280"/>
   </bookViews>
   <sheets>
     <sheet name="questions" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>clue</t>
   </si>
@@ -38,28 +38,34 @@
     <t>keyIndex</t>
   </si>
   <si>
-    <t>Thủ đô Việt Nam</t>
+    <t>1. What system is used to manage courses, students, and learning materials online? (3 letters)</t>
   </si>
   <si>
-    <t>HANOI</t>
+    <t>LMS</t>
   </si>
   <si>
-    <t>Con vật kêu meo</t>
+    <t>2. What is the ability to use digital technologies effectively and responsibly? (15 letters)</t>
   </si>
   <si>
-    <t>MEO</t>
+    <t>DIGITALLITERACY</t>
   </si>
   <si>
-    <t>Trái cây đỏ</t>
+    <t>3. What type of learning uses electronic technologies and the internet? (10 letters)</t>
   </si>
   <si>
-    <t>TAO</t>
+    <t>EELEARNING</t>
   </si>
   <si>
-    <t>Đồ uống sáng</t>
+    <t>4. What refers to storing and managing student or academic data?  (13 letters)</t>
   </si>
   <si>
-    <t>CAFE</t>
+    <t>RECORDKEEPING</t>
+  </si>
+  <si>
+    <t>5. What term describes appropriate behavior when communicating online?(10 letters)</t>
+  </si>
+  <si>
+    <t>NETIQUETTE</t>
   </si>
 </sst>
 </file>
@@ -72,7 +78,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_-* #,##0\ &quot;₫&quot;_-;\-* #,##0\ &quot;₫&quot;_-;_-* &quot;-&quot;\ &quot;₫&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -81,12 +87,23 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Times New Roman"/>
       <charset val="134"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11.25"/>
+      <color rgb="FF081B3A"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -553,144 +570,153 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1226,62 +1252,79 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4" outlineLevelRow="4" outlineLevelCol="2"/>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="13.8" outlineLevelRow="5" outlineLevelCol="2"/>
+  <cols>
+    <col min="1" max="1" width="89.8888888888889" style="1" customWidth="1"/>
+    <col min="2" max="2" width="21.5555555555556" style="1" customWidth="1"/>
+    <col min="3" max="3" width="20.2222222222222" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="10" style="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" ht="28.8" spans="1:3">
-      <c r="A2" s="2" t="s">
+    <row r="2" ht="15" spans="1:3">
+      <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="3" ht="28.8" spans="1:3">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:3">
+      <c r="A3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="2">
-        <v>0</v>
+      <c r="C3" s="5">
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" ht="15" spans="1:3">
+      <c r="A6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="1">
         <v>1</v>
-      </c>
-    </row>
-    <row r="5" ht="28.8" spans="1:3">
-      <c r="A5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="2">
-        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>